<commit_message>
Place supplier images inside detail cells
</commit_message>
<xml_diff>
--- a/plugins/chenyu-kaifa/skills/chenyu-kaifawendang/assets/晨玙产品开发文档母版.xlsx
+++ b/plugins/chenyu-kaifa/skills/chenyu-kaifawendang/assets/晨玙产品开发文档母版.xlsx
@@ -1417,7 +1417,7 @@
       </c>
       <c r="C1" s="22" t="inlineStr">
         <is>
-          <t>供应商产品名称/图片</t>
+          <t>供应商产品图片</t>
         </is>
       </c>
       <c r="D1" s="22" t="inlineStr">
@@ -1436,7 +1436,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1">
+    <row r="2" ht="175" customHeight="1">
       <c r="A2" s="10">
         <f>""</f>
         <v/>
@@ -1462,7 +1462,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="170" customHeight="1">
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" s="10">
         <f>""</f>
         <v/>
@@ -1488,7 +1488,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="175" customHeight="1">
       <c r="A4" s="10">
         <f>""</f>
         <v/>
@@ -1514,7 +1514,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="170" customHeight="1">
+    <row r="5" ht="24" customHeight="1">
       <c r="A5" s="10">
         <f>""</f>
         <v/>
@@ -1540,7 +1540,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="175" customHeight="1">
       <c r="A6" s="10">
         <f>""</f>
         <v/>
@@ -1566,7 +1566,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="170" customHeight="1">
+    <row r="7" ht="24" customHeight="1">
       <c r="A7" s="10">
         <f>""</f>
         <v/>

</xml_diff>